<commit_message>
bd num seq added
</commit_message>
<xml_diff>
--- a/doc/RTL_Bug_Tracking.xlsx
+++ b/doc/RTL_Bug_Tracking.xlsx
@@ -1,13 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\C\ITI\GP\repo\doc\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="4356" windowHeight="4896"/>
   </bookViews>
@@ -20,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="82">
   <si>
     <t>Bug ID</t>
   </si>
@@ -241,12 +236,45 @@
   </si>
   <si>
     <t>15/7/2026</t>
+  </si>
+  <si>
+    <t>RTL_004</t>
+  </si>
+  <si>
+    <t>Nada</t>
+  </si>
+  <si>
+    <t>eth_registers</t>
+  </si>
+  <si>
+    <t>eth_test_reg_access</t>
+  </si>
+  <si>
+    <t>RAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  27/6/2026  </t>
+  </si>
+  <si>
+    <t>MODER bit[11] reserved bit implemented as writable</t>
+  </si>
+  <si>
+    <t>The specification marks MODER bit[11] as reserved, but the DUT allows it to be written/read as an active bit instead of behaving as a reserved bit.</t>
+  </si>
+  <si>
+    <t>tc_01_reg</t>
+  </si>
+  <si>
+    <t>RTL design issue – Reserved bit[11] is not implemented as reserved; writes to the bit are not ignored.</t>
+  </si>
+  <si>
+    <t>MODER Register access</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -280,7 +308,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -316,11 +344,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -350,6 +393,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -362,7 +414,6 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -429,6 +480,249 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
@@ -460,248 +754,6 @@
         </top>
         <bottom style="thin">
           <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
@@ -730,22 +782,22 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BugTable" displayName="BugTable" ref="A1:P4" dataDxfId="16">
   <autoFilter ref="A1:P4"/>
   <tableColumns count="16">
-    <tableColumn id="1" name="Bug ID" dataDxfId="5"/>
-    <tableColumn id="2" name="Date Found" dataDxfId="3"/>
-    <tableColumn id="3" name="Found By" dataDxfId="4"/>
-    <tableColumn id="4" name="Module / Block" dataDxfId="2"/>
-    <tableColumn id="5" name="Feature" dataDxfId="0"/>
-    <tableColumn id="6" name="Bug Summary" dataDxfId="1"/>
-    <tableColumn id="7" name="Detailed Description" dataDxfId="15"/>
-    <tableColumn id="8" name="Severity" dataDxfId="14"/>
-    <tableColumn id="12" name="Test Name" dataDxfId="13"/>
-    <tableColumn id="13" name="Seed" dataDxfId="12"/>
-    <tableColumn id="14" name="Simulation Time" dataDxfId="11"/>
-    <tableColumn id="15" name="Failure Type" dataDxfId="10"/>
-    <tableColumn id="16" name="Waveform Available" dataDxfId="9"/>
-    <tableColumn id="17" name="Root Cause" dataDxfId="8"/>
-    <tableColumn id="21" name="Regression Run" dataDxfId="7"/>
-    <tableColumn id="22" name="Comments" dataDxfId="6"/>
+    <tableColumn id="1" name="Bug ID" dataDxfId="15"/>
+    <tableColumn id="2" name="Date Found" dataDxfId="14"/>
+    <tableColumn id="3" name="Found By" dataDxfId="13"/>
+    <tableColumn id="4" name="Module / Block" dataDxfId="12"/>
+    <tableColumn id="5" name="Feature" dataDxfId="11"/>
+    <tableColumn id="6" name="Bug Summary" dataDxfId="10"/>
+    <tableColumn id="7" name="Detailed Description" dataDxfId="9"/>
+    <tableColumn id="8" name="Severity" dataDxfId="8"/>
+    <tableColumn id="12" name="Test Name" dataDxfId="7"/>
+    <tableColumn id="13" name="Seed" dataDxfId="6"/>
+    <tableColumn id="14" name="Simulation Time" dataDxfId="5"/>
+    <tableColumn id="15" name="Failure Type" dataDxfId="4"/>
+    <tableColumn id="16" name="Waveform Available" dataDxfId="3"/>
+    <tableColumn id="17" name="Root Cause" dataDxfId="2"/>
+    <tableColumn id="21" name="Regression Run" dataDxfId="1"/>
+    <tableColumn id="22" name="Comments" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1036,7 +1088,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.33203125" customWidth="1"/>
@@ -1251,6 +1303,52 @@
       </c>
       <c r="P4" s="5"/>
     </row>
+    <row r="5" spans="1:16" ht="103.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="P5" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1264,19 +1362,19 @@
           <x14:formula1>
             <xm:f>Lists!$A$2:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H501</xm:sqref>
+          <xm:sqref>H2:H4 H6:H501</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list">
           <x14:formula1>
             <xm:f>Lists!$D$2:$D$7</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:L501</xm:sqref>
+          <xm:sqref>L2:L4 L6:L501</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list">
           <x14:formula1>
             <xm:f>Lists!$E$2:$E$3</xm:f>
           </x14:formula1>
-          <xm:sqref>M2:M501</xm:sqref>
+          <xm:sqref>M2:M4 M6:M501</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
added wb_m & tx assertions
</commit_message>
<xml_diff>
--- a/doc/RTL_Bug_Tracking.xlsx
+++ b/doc/RTL_Bug_Tracking.xlsx
@@ -1,8 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\C\ITI\GP\repo\doc\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="4356" windowHeight="4896"/>
   </bookViews>
@@ -15,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="92">
   <si>
     <t>Bug ID</t>
   </si>
@@ -269,12 +274,44 @@
   </si>
   <si>
     <t>MODER Register access</t>
+  </si>
+  <si>
+    <t>RTL_005</t>
+  </si>
+  <si>
+    <t>21/7/2026</t>
+  </si>
+  <si>
+    <t>eth_wishbone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+WB_M - DATA_O - X Propagation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A
+</t>
+  </si>
+  <si>
+    <t>eth_test_tx_smoke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X propagation after Reset assertion </t>
+  </si>
+  <si>
+    <t>tc_01_smoke</t>
+  </si>
+  <si>
+    <t>In wishbone master when reset is asserted, DATA_O is unknown (x)</t>
+  </si>
+  <si>
+    <t>2.5 ns</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -289,7 +326,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -307,8 +344,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -359,48 +402,92 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -414,6 +501,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -480,6 +568,30 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -634,29 +746,6 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -779,25 +868,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BugTable" displayName="BugTable" ref="A1:P4" dataDxfId="16">
-  <autoFilter ref="A1:P4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BugTable" displayName="BugTable" ref="A1:P6" dataDxfId="16">
+  <autoFilter ref="A1:P6"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Bug ID" dataDxfId="15"/>
     <tableColumn id="2" name="Date Found" dataDxfId="14"/>
     <tableColumn id="3" name="Found By" dataDxfId="13"/>
     <tableColumn id="4" name="Module / Block" dataDxfId="12"/>
-    <tableColumn id="5" name="Feature" dataDxfId="11"/>
-    <tableColumn id="6" name="Bug Summary" dataDxfId="10"/>
-    <tableColumn id="7" name="Detailed Description" dataDxfId="9"/>
-    <tableColumn id="8" name="Severity" dataDxfId="8"/>
-    <tableColumn id="12" name="Test Name" dataDxfId="7"/>
-    <tableColumn id="13" name="Seed" dataDxfId="6"/>
-    <tableColumn id="14" name="Simulation Time" dataDxfId="5"/>
-    <tableColumn id="15" name="Failure Type" dataDxfId="4"/>
-    <tableColumn id="16" name="Waveform Available" dataDxfId="3"/>
-    <tableColumn id="17" name="Root Cause" dataDxfId="2"/>
-    <tableColumn id="21" name="Regression Run" dataDxfId="1"/>
-    <tableColumn id="22" name="Comments" dataDxfId="0"/>
+    <tableColumn id="5" name="Feature" dataDxfId="4"/>
+    <tableColumn id="6" name="Bug Summary" dataDxfId="3"/>
+    <tableColumn id="7" name="Detailed Description" dataDxfId="2"/>
+    <tableColumn id="8" name="Severity" dataDxfId="0"/>
+    <tableColumn id="12" name="Test Name" dataDxfId="1"/>
+    <tableColumn id="13" name="Seed" dataDxfId="11"/>
+    <tableColumn id="14" name="Simulation Time" dataDxfId="10"/>
+    <tableColumn id="15" name="Failure Type" dataDxfId="9"/>
+    <tableColumn id="16" name="Waveform Available" dataDxfId="8"/>
+    <tableColumn id="17" name="Root Cause" dataDxfId="7"/>
+    <tableColumn id="21" name="Regression Run" dataDxfId="6"/>
+    <tableColumn id="22" name="Comments" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1088,13 +1177,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.33203125" customWidth="1"/>
     <col min="3" max="3" width="12.21875" customWidth="1"/>
     <col min="4" max="4" width="17.21875" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" customWidth="1"/>
     <col min="6" max="6" width="15.77734375" customWidth="1"/>
     <col min="7" max="7" width="24.77734375" customWidth="1"/>
     <col min="9" max="9" width="19.44140625" customWidth="1"/>
@@ -1157,197 +1246,245 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>61</v>
+      <c r="B2" s="2" t="s">
+        <v>76</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>19</v>
+        <v>73</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="H2" s="21" t="s">
+        <v>32</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="J2" s="2">
-        <v>1</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>22</v>
+        <v>74</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" s="2"/>
+      <c r="L2" s="3" t="s">
+        <v>75</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="N2" s="3" t="s">
-        <v>46</v>
+      <c r="N2" s="8" t="s">
+        <v>80</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>44</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:16" ht="73.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="5">
+        <v>46302</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="L3" s="5" t="s">
+      <c r="E3" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="6">
+        <v>1845683181</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="M3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="P3" s="5"/>
+      <c r="N3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="P3" s="3"/>
     </row>
     <row r="4" spans="1:16" ht="70.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="8">
-        <v>46302</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="J4" s="6">
-        <v>1845683181</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="L4" s="5" t="s">
+      <c r="E4" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" s="12">
+        <v>1</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="L4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="M4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="N4" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="P4" s="5"/>
+      <c r="N4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="O4" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="P4" s="9" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="5" spans="1:16" ht="103.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:16" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="J5" s="4" t="s">
+      <c r="B5" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="M5" s="4" t="s">
+      <c r="L5" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="N5" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="P5" s="4"/>
+      <c r="N5" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="O5" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="P5" s="13"/>
+    </row>
+    <row r="6" spans="1:16" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="J6" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="M6" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="N6" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="O6" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="P6" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1362,19 +1499,19 @@
           <x14:formula1>
             <xm:f>Lists!$A$2:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H4 H6:H501</xm:sqref>
+          <xm:sqref>H3:H6 H8:H501</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list">
           <x14:formula1>
             <xm:f>Lists!$D$2:$D$7</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:L4 L6:L501</xm:sqref>
+          <xm:sqref>L2:L6 L8:L501</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list">
           <x14:formula1>
             <xm:f>Lists!$E$2:$E$3</xm:f>
           </x14:formula1>
-          <xm:sqref>M2:M4 M6:M501</xm:sqref>
+          <xm:sqref>M3:M6 M8:M501</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1384,7 +1521,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -1476,6 +1613,11 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed mdio compile errors
</commit_message>
<xml_diff>
--- a/doc/RTL_Bug_Tracking.xlsx
+++ b/doc/RTL_Bug_Tracking.xlsx
@@ -15,12 +15,12 @@
     <sheet name="Bug_Log" sheetId="1" r:id="rId1"/>
     <sheet name="Lists" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="102">
   <si>
     <t>Bug ID</t>
   </si>
@@ -306,6 +306,37 @@
   </si>
   <si>
     <t>2.5 ns</t>
+  </si>
+  <si>
+    <t>DATA_O is assigned to uninitialized FIFO</t>
+  </si>
+  <si>
+    <t>RTL_006</t>
+  </si>
+  <si>
+    <t>22/7/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+TX - MAXFL </t>
+  </si>
+  <si>
+    <t>Frame is sent when maxfl &lt;=4 bytes</t>
+  </si>
+  <si>
+    <t>eth_test_tx_maxfl</t>
+  </si>
+  <si>
+    <t>tc_10_maxfl</t>
+  </si>
+  <si>
+    <t>Specs states that frames with length = 4bytes or less aren't sent, when maxfl is  4 or less , the configured number is sent and rest of frame is discarded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DUT doesn't check maxfl &gt; 4 bytes </t>
+  </si>
+  <si>
+    <t>eth_txethmac</t>
   </si>
 </sst>
 </file>
@@ -501,7 +532,6 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -524,6 +554,161 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -592,160 +777,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -868,25 +899,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BugTable" displayName="BugTable" ref="A1:P6" dataDxfId="16">
-  <autoFilter ref="A1:P6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BugTable" displayName="BugTable" ref="A1:P7" dataDxfId="16">
+  <autoFilter ref="A1:P7"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Bug ID" dataDxfId="15"/>
     <tableColumn id="2" name="Date Found" dataDxfId="14"/>
     <tableColumn id="3" name="Found By" dataDxfId="13"/>
     <tableColumn id="4" name="Module / Block" dataDxfId="12"/>
-    <tableColumn id="5" name="Feature" dataDxfId="4"/>
-    <tableColumn id="6" name="Bug Summary" dataDxfId="3"/>
-    <tableColumn id="7" name="Detailed Description" dataDxfId="2"/>
-    <tableColumn id="8" name="Severity" dataDxfId="0"/>
-    <tableColumn id="12" name="Test Name" dataDxfId="1"/>
-    <tableColumn id="13" name="Seed" dataDxfId="11"/>
-    <tableColumn id="14" name="Simulation Time" dataDxfId="10"/>
-    <tableColumn id="15" name="Failure Type" dataDxfId="9"/>
-    <tableColumn id="16" name="Waveform Available" dataDxfId="8"/>
-    <tableColumn id="17" name="Root Cause" dataDxfId="7"/>
-    <tableColumn id="21" name="Regression Run" dataDxfId="6"/>
-    <tableColumn id="22" name="Comments" dataDxfId="5"/>
+    <tableColumn id="5" name="Feature" dataDxfId="11"/>
+    <tableColumn id="6" name="Bug Summary" dataDxfId="10"/>
+    <tableColumn id="7" name="Detailed Description" dataDxfId="9"/>
+    <tableColumn id="8" name="Severity" dataDxfId="8"/>
+    <tableColumn id="12" name="Test Name" dataDxfId="7"/>
+    <tableColumn id="13" name="Seed" dataDxfId="6"/>
+    <tableColumn id="14" name="Simulation Time" dataDxfId="5"/>
+    <tableColumn id="15" name="Failure Type" dataDxfId="4"/>
+    <tableColumn id="16" name="Waveform Available" dataDxfId="3"/>
+    <tableColumn id="17" name="Root Cause" dataDxfId="2"/>
+    <tableColumn id="21" name="Regression Run" dataDxfId="1"/>
+    <tableColumn id="22" name="Comments" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1177,7 +1208,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.33203125" customWidth="1"/>
@@ -1185,7 +1216,7 @@
     <col min="4" max="4" width="17.21875" customWidth="1"/>
     <col min="5" max="5" width="11.33203125" customWidth="1"/>
     <col min="6" max="6" width="15.77734375" customWidth="1"/>
-    <col min="7" max="7" width="24.77734375" customWidth="1"/>
+    <col min="7" max="7" width="26.44140625" customWidth="1"/>
     <col min="9" max="9" width="19.44140625" customWidth="1"/>
     <col min="10" max="10" width="11.5546875" customWidth="1"/>
     <col min="11" max="11" width="8.77734375" customWidth="1"/>
@@ -1351,7 +1382,7 @@
         <v>42</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>65</v>
@@ -1425,7 +1456,7 @@
         <v>53</v>
       </c>
       <c r="L5" s="13" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="M5" s="13" t="s">
         <v>23</v>
@@ -1479,12 +1510,60 @@
         <v>23</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="O6" s="13" t="s">
         <v>89</v>
       </c>
       <c r="P6" s="13"/>
+    </row>
+    <row r="7" spans="1:16" ht="70.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="H7" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="K7" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="L7" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="N7" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="O7" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="P7" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1499,19 +1578,19 @@
           <x14:formula1>
             <xm:f>Lists!$A$2:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H6 H8:H501</xm:sqref>
+          <xm:sqref>H3:H501</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list">
           <x14:formula1>
             <xm:f>Lists!$D$2:$D$7</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:L6 L8:L501</xm:sqref>
+          <xm:sqref>L2:L501</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list">
           <x14:formula1>
             <xm:f>Lists!$E$2:$E$3</xm:f>
           </x14:formula1>
-          <xm:sqref>M3:M6 M8:M501</xm:sqref>
+          <xm:sqref>M3:M501</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>